<commit_message>
Separate CI containers and preserve local data
</commit_message>
<xml_diff>
--- a/backend/data/bdd_flux_maf.xlsx
+++ b/backend/data/bdd_flux_maf.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I162"/>
+  <dimension ref="A1:I163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8041,6 +8041,53 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>6379</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>10.20.0.23</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>10.7.1.40</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>SGIC-IAM-QUA-013</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>SG_CACHE</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>outbound</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>API-REST-CRM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>